<commit_message>
final touches to data viz
</commit_message>
<xml_diff>
--- a/data/benthic_monitoring_data.xlsx
+++ b/data/benthic_monitoring_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eac/Documents/GitHub/hhploa/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ec2776/Documents/GitHub/hhlpoa/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA820318-36D4-5E4A-848F-2548E8F71E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A09FEF-EB80-1E41-BEBC-94A2AD4FF9D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4740" yWindow="500" windowWidth="31100" windowHeight="21900" firstSheet="5" activeTab="9" xr2:uid="{31BB1BD1-897F-9B4B-9E56-1AD4E8AE6AD7}"/>
+    <workbookView xWindow="2460" yWindow="660" windowWidth="27780" windowHeight="17280" firstSheet="4" activeTab="10" xr2:uid="{31BB1BD1-897F-9B4B-9E56-1AD4E8AE6AD7}"/>
   </bookViews>
   <sheets>
     <sheet name="Hawk_raw_counts" sheetId="7" r:id="rId1"/>
@@ -25,8 +25,9 @@
     <sheet name="Lake_levels_MinMax" sheetId="14" r:id="rId10"/>
     <sheet name="Diversity_thresholds" sheetId="10" r:id="rId11"/>
     <sheet name="Tolerance_levels" sheetId="6" r:id="rId12"/>
+    <sheet name="min_max_simpsons" sheetId="15" r:id="rId13"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4527" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5018" uniqueCount="168">
   <si>
     <t>Ephemeroptera</t>
   </si>
@@ -528,12 +529,36 @@
   <si>
     <t>Specific_year</t>
   </si>
+  <si>
+    <t>9 groups present</t>
+  </si>
+  <si>
+    <t>sum inds</t>
+  </si>
+  <si>
+    <t>vast majority of individuals (avg 91% were scuds)</t>
+  </si>
+  <si>
+    <t>12 groups present</t>
+  </si>
+  <si>
+    <t>vast majority scuds (avg %85)</t>
+  </si>
+  <si>
+    <t>19 groups present</t>
+  </si>
+  <si>
+    <t>site_name</t>
+  </si>
+  <si>
+    <t>number</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -579,13 +604,44 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -600,7 +656,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -621,9 +677,20 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="22" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9500,40 +9567,40 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="6" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="14">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6">
         <v>2013</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="14" t="s">
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
         <v>156</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="14">
         <v>41286.341134259259</v>
       </c>
       <c r="E6" s="12">
         <v>2.1671044265592601</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="14">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7">
         <v>2013</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="14" t="s">
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
         <v>157</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="14">
         <v>41390.370520833334</v>
       </c>
       <c r="E7" s="12">
         <v>4.85253030063026</v>
       </c>
-      <c r="G7" s="16"/>
+      <c r="G7" s="15"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8">
@@ -10583,8 +10650,8 @@
       <c r="F14">
         <v>3.75</v>
       </c>
-      <c r="G14" t="s">
-        <v>129</v>
+      <c r="G14" s="23" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -10606,8 +10673,8 @@
       <c r="F15">
         <v>4.25</v>
       </c>
-      <c r="G15" t="s">
-        <v>125</v>
+      <c r="G15" s="23" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -10629,8 +10696,8 @@
       <c r="F16">
         <v>5</v>
       </c>
-      <c r="G16" t="s">
-        <v>130</v>
+      <c r="G16" s="23" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -10652,7 +10719,7 @@
       <c r="F17">
         <v>5.75</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="23" t="s">
         <v>126</v>
       </c>
     </row>
@@ -10675,8 +10742,8 @@
       <c r="F18">
         <v>6.5</v>
       </c>
-      <c r="G18" t="s">
-        <v>127</v>
+      <c r="G18" s="23" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -10698,8 +10765,8 @@
       <c r="F19">
         <v>7.25</v>
       </c>
-      <c r="G19" t="s">
-        <v>131</v>
+      <c r="G19" s="23" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -10721,8 +10788,8 @@
       <c r="F20">
         <v>10</v>
       </c>
-      <c r="G20" t="s">
-        <v>128</v>
+      <c r="G20" s="23" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -10744,8 +10811,8 @@
       <c r="F21">
         <v>3.75</v>
       </c>
-      <c r="G21" t="s">
-        <v>129</v>
+      <c r="G21" s="23" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -10767,8 +10834,8 @@
       <c r="F22">
         <v>4.25</v>
       </c>
-      <c r="G22" t="s">
-        <v>125</v>
+      <c r="G22" s="23" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -10790,8 +10857,8 @@
       <c r="F23">
         <v>5</v>
       </c>
-      <c r="G23" t="s">
-        <v>130</v>
+      <c r="G23" s="23" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -10813,7 +10880,7 @@
       <c r="F24">
         <v>5.75</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24" s="23" t="s">
         <v>126</v>
       </c>
     </row>
@@ -10836,8 +10903,8 @@
       <c r="F25">
         <v>6.5</v>
       </c>
-      <c r="G25" t="s">
-        <v>127</v>
+      <c r="G25" s="23" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -10859,8 +10926,8 @@
       <c r="F26">
         <v>7.25</v>
       </c>
-      <c r="G26" t="s">
-        <v>131</v>
+      <c r="G26" s="23" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -10882,8 +10949,8 @@
       <c r="F27">
         <v>10</v>
       </c>
-      <c r="G27" t="s">
-        <v>128</v>
+      <c r="G27" s="23" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -10905,8 +10972,8 @@
       <c r="F28">
         <v>3.75</v>
       </c>
-      <c r="G28" t="s">
-        <v>129</v>
+      <c r="G28" s="23" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -10928,8 +10995,8 @@
       <c r="F29">
         <v>4.25</v>
       </c>
-      <c r="G29" t="s">
-        <v>125</v>
+      <c r="G29" s="23" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
@@ -10951,8 +11018,8 @@
       <c r="F30">
         <v>5</v>
       </c>
-      <c r="G30" t="s">
-        <v>130</v>
+      <c r="G30" s="23" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -10974,7 +11041,7 @@
       <c r="F31">
         <v>5.75</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" s="23" t="s">
         <v>126</v>
       </c>
     </row>
@@ -10997,8 +11064,8 @@
       <c r="F32">
         <v>6.5</v>
       </c>
-      <c r="G32" t="s">
-        <v>127</v>
+      <c r="G32" s="23" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -11020,8 +11087,8 @@
       <c r="F33">
         <v>7.25</v>
       </c>
-      <c r="G33" t="s">
-        <v>131</v>
+      <c r="G33" s="23" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -11043,8 +11110,8 @@
       <c r="F34">
         <v>10</v>
       </c>
-      <c r="G34" t="s">
-        <v>128</v>
+      <c r="G34" s="23" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -11581,6 +11648,2778 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C28">
     <sortCondition ref="C2:C28"/>
   </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD388846-98A4-C34F-A55E-75EB16FA8853}">
+  <dimension ref="A1:Z88"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A2" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E2" s="16">
+        <v>0</v>
+      </c>
+      <c r="F2" s="16">
+        <v>0</v>
+      </c>
+      <c r="G2" s="16"/>
+      <c r="H2">
+        <v>2021</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" t="s">
+        <v>61</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>2022</v>
+      </c>
+      <c r="P2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>33</v>
+      </c>
+      <c r="R2" t="s">
+        <v>61</v>
+      </c>
+      <c r="S2" s="2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A3" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E3" s="16">
+        <v>0</v>
+      </c>
+      <c r="F3" s="16">
+        <v>0</v>
+      </c>
+      <c r="G3" s="16"/>
+      <c r="H3">
+        <v>2021</v>
+      </c>
+      <c r="I3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" t="s">
+        <v>96</v>
+      </c>
+      <c r="K3" t="s">
+        <v>62</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="O3" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P3" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q3" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="R3" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="S3" s="22">
+        <v>3</v>
+      </c>
+      <c r="T3" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A4" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="E4" s="16">
+        <v>0</v>
+      </c>
+      <c r="F4" s="16">
+        <v>0</v>
+      </c>
+      <c r="G4" s="16"/>
+      <c r="H4">
+        <v>2021</v>
+      </c>
+      <c r="I4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" t="s">
+        <v>97</v>
+      </c>
+      <c r="K4" t="s">
+        <v>63</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="O4" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P4" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q4" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="R4" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="S4" s="22">
+        <v>1</v>
+      </c>
+      <c r="T4" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A5" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" s="16">
+        <v>0</v>
+      </c>
+      <c r="F5" s="16">
+        <v>0</v>
+      </c>
+      <c r="G5" s="16"/>
+      <c r="H5">
+        <v>2021</v>
+      </c>
+      <c r="I5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" t="s">
+        <v>98</v>
+      </c>
+      <c r="K5" t="s">
+        <v>64</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="O5" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P5" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q5" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="R5" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="S5" s="22">
+        <v>3</v>
+      </c>
+      <c r="T5" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A6" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" s="16">
+        <v>0</v>
+      </c>
+      <c r="F6" s="16">
+        <v>0</v>
+      </c>
+      <c r="G6" s="16"/>
+      <c r="H6" s="20">
+        <v>2021</v>
+      </c>
+      <c r="I6" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="K6" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="L6" s="20">
+        <v>0</v>
+      </c>
+      <c r="M6" s="20">
+        <v>1</v>
+      </c>
+      <c r="O6">
+        <v>2022</v>
+      </c>
+      <c r="P6" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>42</v>
+      </c>
+      <c r="R6" t="s">
+        <v>65</v>
+      </c>
+      <c r="S6" s="2">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A7" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" s="16">
+        <v>0</v>
+      </c>
+      <c r="F7" s="16">
+        <v>0</v>
+      </c>
+      <c r="G7" s="16"/>
+      <c r="H7" s="20">
+        <v>2021</v>
+      </c>
+      <c r="I7" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="J7" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="K7" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="L7" s="20">
+        <v>4</v>
+      </c>
+      <c r="M7" s="20">
+        <v>0</v>
+      </c>
+      <c r="O7" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P7" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q7" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="R7" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="S7" s="22">
+        <v>22</v>
+      </c>
+      <c r="T7" s="21">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A8" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" s="16">
+        <v>0</v>
+      </c>
+      <c r="F8" s="16">
+        <v>0</v>
+      </c>
+      <c r="G8" s="16"/>
+      <c r="H8" s="20">
+        <v>2021</v>
+      </c>
+      <c r="I8" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="J8" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="K8" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="L8" s="20">
+        <v>2</v>
+      </c>
+      <c r="M8" s="20">
+        <v>0</v>
+      </c>
+      <c r="O8" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P8" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q8" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="R8" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="S8" s="22">
+        <v>1</v>
+      </c>
+      <c r="T8" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A9" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="E9" s="18">
+        <v>100</v>
+      </c>
+      <c r="F9" s="18">
+        <v>91</v>
+      </c>
+      <c r="G9" s="16"/>
+      <c r="H9" s="20">
+        <v>2021</v>
+      </c>
+      <c r="I9" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="J9" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="K9" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="L9" s="20">
+        <v>168</v>
+      </c>
+      <c r="M9" s="20">
+        <v>163</v>
+      </c>
+      <c r="O9" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P9" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q9" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="R9" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="S9" s="22">
+        <v>19</v>
+      </c>
+      <c r="T9" s="21">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A10" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="E10" s="16">
+        <v>0</v>
+      </c>
+      <c r="F10" s="16">
+        <v>0</v>
+      </c>
+      <c r="G10" s="16"/>
+      <c r="H10">
+        <v>2021</v>
+      </c>
+      <c r="I10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J10" t="s">
+        <v>44</v>
+      </c>
+      <c r="K10" t="s">
+        <v>69</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>2022</v>
+      </c>
+      <c r="P10" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>44</v>
+      </c>
+      <c r="R10" t="s">
+        <v>69</v>
+      </c>
+      <c r="S10" s="2">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A11" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="18">
+        <v>0</v>
+      </c>
+      <c r="F11" s="18">
+        <v>1</v>
+      </c>
+      <c r="G11" s="16"/>
+      <c r="H11">
+        <v>2021</v>
+      </c>
+      <c r="I11" t="s">
+        <v>17</v>
+      </c>
+      <c r="J11" t="s">
+        <v>100</v>
+      </c>
+      <c r="K11" t="s">
+        <v>70</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>2022</v>
+      </c>
+      <c r="P11" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>100</v>
+      </c>
+      <c r="R11" t="s">
+        <v>70</v>
+      </c>
+      <c r="S11" s="2">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A12" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" s="18">
+        <v>0</v>
+      </c>
+      <c r="F12" s="18">
+        <v>1</v>
+      </c>
+      <c r="G12" s="16"/>
+      <c r="H12" s="20">
+        <v>2021</v>
+      </c>
+      <c r="I12" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="J12" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="K12" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="L12" s="20">
+        <v>5</v>
+      </c>
+      <c r="M12" s="20">
+        <v>6</v>
+      </c>
+      <c r="O12" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P12" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q12" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="R12" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="S12" s="22">
+        <v>3</v>
+      </c>
+      <c r="T12" s="21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A13" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="16">
+        <v>0</v>
+      </c>
+      <c r="F13" s="16">
+        <v>0</v>
+      </c>
+      <c r="G13" s="16"/>
+      <c r="H13" s="20">
+        <v>2021</v>
+      </c>
+      <c r="I13" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="J13" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="K13" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="L13" s="20">
+        <v>0</v>
+      </c>
+      <c r="M13" s="20">
+        <v>1</v>
+      </c>
+      <c r="O13" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P13" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q13" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="R13" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="S13" s="22">
+        <v>12</v>
+      </c>
+      <c r="T13" s="21">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A14" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E14" s="18">
+        <v>0</v>
+      </c>
+      <c r="F14" s="18">
+        <v>2</v>
+      </c>
+      <c r="G14" s="16"/>
+      <c r="H14">
+        <v>2021</v>
+      </c>
+      <c r="I14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J14" t="s">
+        <v>2</v>
+      </c>
+      <c r="K14" t="s">
+        <v>73</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="O14" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P14" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q14" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="R14" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="S14" s="22">
+        <v>5</v>
+      </c>
+      <c r="T14" s="21">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A15" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15" s="16">
+        <v>0</v>
+      </c>
+      <c r="F15" s="16">
+        <v>0</v>
+      </c>
+      <c r="G15" s="16"/>
+      <c r="H15">
+        <v>2021</v>
+      </c>
+      <c r="I15" t="s">
+        <v>17</v>
+      </c>
+      <c r="J15" t="s">
+        <v>101</v>
+      </c>
+      <c r="K15" t="s">
+        <v>74</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="O15" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P15" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q15" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="R15" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="S15" s="22">
+        <v>1</v>
+      </c>
+      <c r="T15" s="21">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A16" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="E16" s="18">
+        <v>0</v>
+      </c>
+      <c r="F16" s="18">
+        <v>1</v>
+      </c>
+      <c r="G16" s="16"/>
+      <c r="H16">
+        <v>2021</v>
+      </c>
+      <c r="I16" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" t="s">
+        <v>45</v>
+      </c>
+      <c r="K16" t="s">
+        <v>75</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>2022</v>
+      </c>
+      <c r="P16" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>45</v>
+      </c>
+      <c r="R16" t="s">
+        <v>75</v>
+      </c>
+      <c r="S16" s="2">
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A17" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" s="16">
+        <v>0</v>
+      </c>
+      <c r="F17" s="16">
+        <v>0</v>
+      </c>
+      <c r="G17" s="16"/>
+      <c r="H17" s="20">
+        <v>2021</v>
+      </c>
+      <c r="I17" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="J17" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="K17" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="L17" s="20">
+        <v>2</v>
+      </c>
+      <c r="M17" s="20">
+        <v>2</v>
+      </c>
+      <c r="O17" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P17" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q17" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="R17" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="S17" s="22">
+        <v>5</v>
+      </c>
+      <c r="T17" s="21">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A18" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="18">
+        <v>0</v>
+      </c>
+      <c r="F18" s="18">
+        <v>1</v>
+      </c>
+      <c r="G18" s="16"/>
+      <c r="H18" s="20">
+        <v>2021</v>
+      </c>
+      <c r="I18" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="J18" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="K18" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="L18" s="20">
+        <v>10</v>
+      </c>
+      <c r="M18" s="20">
+        <v>1</v>
+      </c>
+      <c r="O18" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P18" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q18" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="R18" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="S18" s="22">
+        <v>0</v>
+      </c>
+      <c r="T18" s="21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A19" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E19" s="16">
+        <v>0</v>
+      </c>
+      <c r="F19" s="16">
+        <v>0</v>
+      </c>
+      <c r="G19" s="16"/>
+      <c r="H19">
+        <v>2021</v>
+      </c>
+      <c r="I19" t="s">
+        <v>17</v>
+      </c>
+      <c r="J19" t="s">
+        <v>46</v>
+      </c>
+      <c r="K19" t="s">
+        <v>78</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>2022</v>
+      </c>
+      <c r="P19" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>46</v>
+      </c>
+      <c r="R19" t="s">
+        <v>78</v>
+      </c>
+      <c r="S19" s="2">
+        <v>0</v>
+      </c>
+      <c r="T19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A20" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" s="18">
+        <v>1</v>
+      </c>
+      <c r="F20" s="18">
+        <v>0</v>
+      </c>
+      <c r="G20" s="16"/>
+      <c r="H20" s="20">
+        <v>2021</v>
+      </c>
+      <c r="I20" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="J20" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="K20" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="L20" s="20">
+        <v>1</v>
+      </c>
+      <c r="M20" s="20">
+        <v>0</v>
+      </c>
+      <c r="O20">
+        <v>2022</v>
+      </c>
+      <c r="P20" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>41</v>
+      </c>
+      <c r="R20" t="s">
+        <v>79</v>
+      </c>
+      <c r="S20" s="2">
+        <v>0</v>
+      </c>
+      <c r="T20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A21" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="E21" s="18">
+        <v>1</v>
+      </c>
+      <c r="F21" s="18">
+        <v>0</v>
+      </c>
+      <c r="G21" s="16"/>
+      <c r="H21" s="20">
+        <v>2021</v>
+      </c>
+      <c r="I21" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="J21" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="K21" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="L21" s="20">
+        <v>10</v>
+      </c>
+      <c r="M21" s="20">
+        <v>2</v>
+      </c>
+      <c r="O21" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P21" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q21" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="R21" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="S21" s="22">
+        <v>13</v>
+      </c>
+      <c r="T21" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A22" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="E22" s="18">
+        <v>5</v>
+      </c>
+      <c r="F22" s="18">
+        <v>6</v>
+      </c>
+      <c r="G22" s="16"/>
+      <c r="H22" s="20">
+        <v>2021</v>
+      </c>
+      <c r="I22" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="J22" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="K22" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="L22" s="20">
+        <v>7</v>
+      </c>
+      <c r="M22" s="20">
+        <v>4</v>
+      </c>
+      <c r="O22" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P22" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q22" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="R22" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="S22" s="22">
+        <v>1</v>
+      </c>
+      <c r="T22" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A23" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="E23" s="16">
+        <v>0</v>
+      </c>
+      <c r="F23" s="16">
+        <v>0</v>
+      </c>
+      <c r="G23" s="16"/>
+      <c r="H23">
+        <v>2021</v>
+      </c>
+      <c r="I23" t="s">
+        <v>17</v>
+      </c>
+      <c r="J23" t="s">
+        <v>47</v>
+      </c>
+      <c r="K23" t="s">
+        <v>82</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="O23" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P23" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q23" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="R23" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="S23" s="22">
+        <v>1</v>
+      </c>
+      <c r="T23" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A24" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="E24" s="16">
+        <v>0</v>
+      </c>
+      <c r="F24" s="16">
+        <v>0</v>
+      </c>
+      <c r="G24" s="16"/>
+      <c r="H24">
+        <v>2021</v>
+      </c>
+      <c r="I24" t="s">
+        <v>17</v>
+      </c>
+      <c r="J24" t="s">
+        <v>48</v>
+      </c>
+      <c r="K24" t="s">
+        <v>83</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24">
+        <v>0</v>
+      </c>
+      <c r="O24" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P24" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q24" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="R24" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="S24" s="22">
+        <v>1</v>
+      </c>
+      <c r="T24" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A25" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="E25" s="16">
+        <v>0</v>
+      </c>
+      <c r="F25" s="16">
+        <v>0</v>
+      </c>
+      <c r="G25" s="16"/>
+      <c r="H25" s="20">
+        <v>2021</v>
+      </c>
+      <c r="I25" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="J25" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="K25" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="L25" s="20">
+        <v>5</v>
+      </c>
+      <c r="M25" s="20">
+        <v>0</v>
+      </c>
+      <c r="O25" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P25" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q25" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="R25" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="S25" s="22">
+        <v>3</v>
+      </c>
+      <c r="T25" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A26" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="E26" s="16">
+        <v>0</v>
+      </c>
+      <c r="F26" s="16">
+        <v>0</v>
+      </c>
+      <c r="G26" s="16"/>
+      <c r="H26">
+        <v>2021</v>
+      </c>
+      <c r="I26" t="s">
+        <v>17</v>
+      </c>
+      <c r="J26" t="s">
+        <v>102</v>
+      </c>
+      <c r="K26" t="s">
+        <v>85</v>
+      </c>
+      <c r="L26">
+        <v>0</v>
+      </c>
+      <c r="M26">
+        <v>0</v>
+      </c>
+      <c r="O26" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P26" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q26" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="R26" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="S26" s="22">
+        <v>1</v>
+      </c>
+      <c r="T26" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A27" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="E27" s="16">
+        <v>0</v>
+      </c>
+      <c r="F27" s="16">
+        <v>0</v>
+      </c>
+      <c r="G27" s="16"/>
+      <c r="H27">
+        <v>2021</v>
+      </c>
+      <c r="I27" t="s">
+        <v>17</v>
+      </c>
+      <c r="J27" t="s">
+        <v>103</v>
+      </c>
+      <c r="K27" t="s">
+        <v>86</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27">
+        <v>0</v>
+      </c>
+      <c r="O27">
+        <v>2022</v>
+      </c>
+      <c r="P27" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>103</v>
+      </c>
+      <c r="R27" t="s">
+        <v>86</v>
+      </c>
+      <c r="S27" s="2">
+        <v>0</v>
+      </c>
+      <c r="T27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A28" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="E28" s="16">
+        <v>0</v>
+      </c>
+      <c r="F28" s="16">
+        <v>0</v>
+      </c>
+      <c r="G28" s="16"/>
+      <c r="H28">
+        <v>2021</v>
+      </c>
+      <c r="I28" t="s">
+        <v>17</v>
+      </c>
+      <c r="J28" t="s">
+        <v>104</v>
+      </c>
+      <c r="K28" t="s">
+        <v>87</v>
+      </c>
+      <c r="L28">
+        <v>0</v>
+      </c>
+      <c r="M28">
+        <v>0</v>
+      </c>
+      <c r="O28" s="21">
+        <v>2022</v>
+      </c>
+      <c r="P28" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q28" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="R28" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="S28" s="22">
+        <v>6</v>
+      </c>
+      <c r="T28" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="D29" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="E29" s="1">
+        <f>SUM(E2:E28)</f>
+        <v>107</v>
+      </c>
+      <c r="F29" s="1">
+        <f>SUM(F2:F28)</f>
+        <v>103</v>
+      </c>
+      <c r="K29" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="L29" s="1">
+        <f>SUM(L2:L28)</f>
+        <v>214</v>
+      </c>
+      <c r="M29" s="1">
+        <f>SUM(M2:M28)</f>
+        <v>180</v>
+      </c>
+      <c r="R29" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="S29" s="1">
+        <f>SUM(S2:S28)</f>
+        <v>101</v>
+      </c>
+      <c r="T29" s="1">
+        <f>SUM(T2:T28)</f>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="D31" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="R31" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="D32" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C35" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E35" s="16">
+        <v>0</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E36" s="16">
+        <v>0</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="E37" s="16">
+        <v>0</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E38" s="16">
+        <v>0</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A39" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="E39" s="16">
+        <v>0</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A40" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B40" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E40" s="16">
+        <v>0</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A41" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B41" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E41" s="16">
+        <v>0</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A42" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B42" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="D42" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="E42" s="18">
+        <v>100</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A43" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="E43" s="16">
+        <v>0</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B44" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C44" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="D44" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="E44" s="18">
+        <v>0</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A45" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B45" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C45" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="D45" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="E45" s="18">
+        <v>0</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A46" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B46" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C46" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E46" s="16">
+        <v>0</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B47" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C47" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D47" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E47" s="18">
+        <v>0</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A48" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B48" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C48" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="E48" s="16">
+        <v>0</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A49" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B49" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C49" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D49" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="E49" s="18">
+        <v>0</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A50" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D50" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E50" s="16">
+        <v>0</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A51" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B51" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C51" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="D51" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="E51" s="18">
+        <v>0</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A52" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B52" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C52" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D52" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E52" s="16">
+        <v>0</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A53" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B53" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C53" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D53" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="E53" s="18">
+        <v>1</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A54" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B54" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C54" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="D54" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="E54" s="18">
+        <v>1</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A55" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B55" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C55" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="D55" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="E55" s="18">
+        <v>5</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A56" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B56" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="D56" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="E56" s="16">
+        <v>0</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A57" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B57" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C57" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="E57" s="16">
+        <v>0</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A58" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B58" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C58" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D58" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="E58" s="16">
+        <v>0</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A59" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B59" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C59" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="D59" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="E59" s="16">
+        <v>0</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A60" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B60" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C60" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D60" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="E60" s="16">
+        <v>0</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A61" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B61" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C61" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D61" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="E61" s="16">
+        <v>0</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A62">
+        <v>2022</v>
+      </c>
+      <c r="B62" t="s">
+        <v>17</v>
+      </c>
+      <c r="C62" t="s">
+        <v>33</v>
+      </c>
+      <c r="D62" t="s">
+        <v>61</v>
+      </c>
+      <c r="E62" s="2">
+        <v>0</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A63" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B63" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C63" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="D63" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="E63" s="22">
+        <v>3</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A64" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B64" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C64" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="D64" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="E64" s="22">
+        <v>1</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A65" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B65" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C65" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="D65" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="E65" s="22">
+        <v>3</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>2022</v>
+      </c>
+      <c r="B66" t="s">
+        <v>17</v>
+      </c>
+      <c r="C66" t="s">
+        <v>42</v>
+      </c>
+      <c r="D66" t="s">
+        <v>65</v>
+      </c>
+      <c r="E66" s="2">
+        <v>0</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A67" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B67" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C67" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="D67" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="E67" s="22">
+        <v>22</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A68" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B68" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C68" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D68" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="E68" s="22">
+        <v>1</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A69" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B69" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C69" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="D69" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="E69" s="22">
+        <v>19</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>2022</v>
+      </c>
+      <c r="B70" t="s">
+        <v>17</v>
+      </c>
+      <c r="C70" t="s">
+        <v>44</v>
+      </c>
+      <c r="D70" t="s">
+        <v>69</v>
+      </c>
+      <c r="E70" s="2">
+        <v>0</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>2022</v>
+      </c>
+      <c r="B71" t="s">
+        <v>17</v>
+      </c>
+      <c r="C71" t="s">
+        <v>100</v>
+      </c>
+      <c r="D71" t="s">
+        <v>70</v>
+      </c>
+      <c r="E71" s="2">
+        <v>0</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A72" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B72" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C72" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="D72" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="E72" s="22">
+        <v>3</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A73" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B73" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C73" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="D73" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="E73" s="22">
+        <v>12</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A74" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B74" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C74" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="D74" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E74" s="22">
+        <v>5</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A75" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B75" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C75" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="D75" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="E75" s="22">
+        <v>1</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A76">
+        <v>2022</v>
+      </c>
+      <c r="B76" t="s">
+        <v>17</v>
+      </c>
+      <c r="C76" t="s">
+        <v>45</v>
+      </c>
+      <c r="D76" t="s">
+        <v>75</v>
+      </c>
+      <c r="E76" s="2">
+        <v>0</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A77" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B77" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C77" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D77" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="E77" s="22">
+        <v>5</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A78" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B78" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C78" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="D78" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="E78" s="22">
+        <v>0</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A79">
+        <v>2022</v>
+      </c>
+      <c r="B79" t="s">
+        <v>17</v>
+      </c>
+      <c r="C79" t="s">
+        <v>46</v>
+      </c>
+      <c r="D79" t="s">
+        <v>78</v>
+      </c>
+      <c r="E79" s="2">
+        <v>0</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A80">
+        <v>2022</v>
+      </c>
+      <c r="B80" t="s">
+        <v>17</v>
+      </c>
+      <c r="C80" t="s">
+        <v>41</v>
+      </c>
+      <c r="D80" t="s">
+        <v>79</v>
+      </c>
+      <c r="E80" s="2">
+        <v>0</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A81" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B81" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C81" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="D81" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="E81" s="22">
+        <v>13</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A82" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B82" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C82" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="D82" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="E82" s="22">
+        <v>1</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A83" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B83" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C83" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="D83" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="E83" s="22">
+        <v>1</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A84" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B84" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C84" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D84" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="E84" s="22">
+        <v>1</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A85" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B85" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C85" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D85" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="E85" s="22">
+        <v>3</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A86" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B86" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C86" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="D86" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="E86" s="22">
+        <v>1</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A87">
+        <v>2022</v>
+      </c>
+      <c r="B87" t="s">
+        <v>17</v>
+      </c>
+      <c r="C87" t="s">
+        <v>103</v>
+      </c>
+      <c r="D87" t="s">
+        <v>86</v>
+      </c>
+      <c r="E87" s="2">
+        <v>0</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A88" s="21">
+        <v>2022</v>
+      </c>
+      <c r="B88" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C88" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="D88" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E88" s="22">
+        <v>6</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>